<commit_message>
Auto-create test data folders in create_input_map
</commit_message>
<xml_diff>
--- a/input/input_map.xlsx
+++ b/input/input_map.xlsx
@@ -24,12 +24,18 @@
     <sheet name="Manual Scavanger Certificate" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="Vulnerable Tribal Certificate" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="Bonded Labour Certificate" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="Single Mother Certificate" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="Bank Passbook" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="General Caste Self Decl" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="Institute Affiliation Decl" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="Orphan Certificate" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="Ration Card" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="BOC Certificate" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Single Mother Certificate" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="Bank Passbook" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="General Caste Self Decl" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="Institute Affiliation Decl" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="Orphan Certificate" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="Ration Card" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="Divyang Certificate" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="Occupation Certificate" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="Annual Contribution Certificate" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="Transgender Certificate" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="Visa" sheetId="29" state="visible" r:id="rId29"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -39,7 +45,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="24">
+  <fonts count="25">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -156,6 +162,18 @@
     <font>
       <name val="Calibri"/>
       <i val="1"/>
+      <color rgb="00283593"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00AAAAAA"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
       <color rgb="0001579B"/>
       <sz val="10"/>
     </font>
@@ -163,12 +181,6 @@
       <name val="Calibri"/>
       <i val="1"/>
       <color rgb="00F9A825"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <i val="1"/>
-      <color rgb="00283593"/>
       <sz val="10"/>
     </font>
     <font>
@@ -288,17 +300,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00E8EAF6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FFF3E0"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E1F5FE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E8EAF6"/>
       </patternFill>
     </fill>
     <fill>
@@ -325,7 +337,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -486,8 +498,11 @@
     <xf numFmtId="0" fontId="3" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -495,7 +510,7 @@
     <xf numFmtId="0" fontId="3" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="22" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="22" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -503,9 +518,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="22" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -516,10 +528,13 @@
     <xf numFmtId="0" fontId="3" fillId="23" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="24" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -527,6 +542,21 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="24" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2585,6 +2615,199 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00E8EAF6"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="65" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="36" customHeight="1">
+      <c r="A1" s="54" t="inlineStr">
+        <is>
+          <t>Paste full file paths in Column A (JPG / PNG / PDF). Column B = optional notes. Column C = Run Status (auto-updated by script). All files in this sheet = BOC Certificate</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>File Path</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Notes (optional)</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Run Status</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Output Row</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="55" t="inlineStr">
+        <is>
+          <t>&lt;path to BOC Certificate file 1&gt;</t>
+        </is>
+      </c>
+      <c r="B3" s="56" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D3" s="57" t="inlineStr"/>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="55" t="inlineStr">
+        <is>
+          <t>&lt;path to BOC Certificate file 2&gt;</t>
+        </is>
+      </c>
+      <c r="B4" s="56" t="inlineStr"/>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D4" s="57" t="inlineStr"/>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="55" t="inlineStr">
+        <is>
+          <t>&lt;path to BOC Certificate file 3&gt;</t>
+        </is>
+      </c>
+      <c r="B5" s="56" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D5" s="57" t="inlineStr"/>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="55" t="inlineStr">
+        <is>
+          <t>&lt;path to BOC Certificate file 4&gt;</t>
+        </is>
+      </c>
+      <c r="B6" s="56" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D6" s="57" t="inlineStr"/>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="55" t="inlineStr">
+        <is>
+          <t>&lt;path to BOC Certificate file 5&gt;</t>
+        </is>
+      </c>
+      <c r="B7" s="56" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D7" s="57" t="inlineStr"/>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="55" t="inlineStr">
+        <is>
+          <t>&lt;path to BOC Certificate file 6&gt;</t>
+        </is>
+      </c>
+      <c r="B8" s="56" t="inlineStr"/>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D8" s="57" t="inlineStr"/>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="55" t="inlineStr">
+        <is>
+          <t>&lt;path to BOC Certificate file 7&gt;</t>
+        </is>
+      </c>
+      <c r="B9" s="56" t="inlineStr"/>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D9" s="57" t="inlineStr"/>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="55" t="inlineStr">
+        <is>
+          <t>&lt;path to BOC Certificate file 8&gt;</t>
+        </is>
+      </c>
+      <c r="B10" s="56" t="inlineStr"/>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D10" s="57" t="inlineStr"/>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="55" t="inlineStr">
+        <is>
+          <t>&lt;path to BOC Certificate file 9&gt;</t>
+        </is>
+      </c>
+      <c r="B11" s="56" t="inlineStr"/>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D11" s="57" t="inlineStr"/>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="55" t="inlineStr">
+        <is>
+          <t>&lt;path to BOC Certificate file 10&gt;</t>
+        </is>
+      </c>
+      <c r="B12" s="56" t="inlineStr"/>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D12" s="57" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="00FFF3E0"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -2599,7 +2822,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
-      <c r="A1" s="54" t="inlineStr">
+      <c r="A1" s="58" t="inlineStr">
         <is>
           <t>Paste full file paths in Column A (JPG / PNG / PDF). Column B = optional notes. Column C = Run Status (auto-updated by script). All files in this sheet = Single Mother Certificate</t>
         </is>
@@ -2628,99 +2851,18 @@
       </c>
     </row>
     <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="55" t="inlineStr">
+      <c r="A3" s="59" t="inlineStr">
         <is>
           <t>D:\ai_doc_automation\Test Data\Single Mother Certificate for Testing\Single Mother Certificate.pdf</t>
         </is>
       </c>
-      <c r="B3" s="56" t="inlineStr"/>
+      <c r="B3" s="60" t="inlineStr"/>
       <c r="C3" s="5" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
       </c>
-      <c r="D3" s="56" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="00E1F5FE"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="65" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="36" customHeight="1">
-      <c r="A1" s="57" t="inlineStr">
-        <is>
-          <t>Paste full file paths in Column A (JPG / PNG / PDF). Column B = optional notes. Column C = Run Status (auto-updated by script). All files in this sheet = Bank Passbook</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>File Path</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Notes (optional)</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Run Status</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Output Row</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="58" t="inlineStr">
-        <is>
-          <t>D:\ai_doc_automation\Test Data\Bank Passbook for Testing\1.webp</t>
-        </is>
-      </c>
-      <c r="B3" s="59" t="inlineStr"/>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="D3" s="59" t="inlineStr"/>
-    </row>
-    <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="58" t="inlineStr">
-        <is>
-          <t>D:\ai_doc_automation\Test Data\Bank Passbook for Testing\Pass book.pdf</t>
-        </is>
-      </c>
-      <c r="B4" s="59" t="inlineStr"/>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="D4" s="59" t="inlineStr"/>
+      <c r="D3" s="60" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2856,6 +2998,87 @@
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00E1F5FE"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="65" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="36" customHeight="1">
+      <c r="A1" s="61" t="inlineStr">
+        <is>
+          <t>Paste full file paths in Column A (JPG / PNG / PDF). Column B = optional notes. Column C = Run Status (auto-updated by script). All files in this sheet = Bank Passbook</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>File Path</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Notes (optional)</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Run Status</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Output Row</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="62" t="inlineStr">
+        <is>
+          <t>D:\ai_doc_automation\Test Data\Bank Passbook for Testing\1.webp</t>
+        </is>
+      </c>
+      <c r="B3" s="63" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D3" s="63" t="inlineStr"/>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="62" t="inlineStr">
+        <is>
+          <t>D:\ai_doc_automation\Test Data\Bank Passbook for Testing\Pass book.pdf</t>
+        </is>
+      </c>
+      <c r="B4" s="63" t="inlineStr"/>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D4" s="63" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="00FFF8E1"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -2870,7 +3093,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
-      <c r="A1" s="60" t="inlineStr">
+      <c r="A1" s="64" t="inlineStr">
         <is>
           <t>Paste full file paths in Column A (JPG / PNG / PDF). Column B = optional notes. Column C = Run Status (auto-updated by script). All files in this sheet = General Caste Self Decl</t>
         </is>
@@ -2920,7 +3143,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00E8EAF6"/>
@@ -2937,7 +3160,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
-      <c r="A1" s="61" t="inlineStr">
+      <c r="A1" s="54" t="inlineStr">
         <is>
           <t>Paste full file paths in Column A (JPG / PNG / PDF). Column B = optional notes. Column C = Run Status (auto-updated by script). All files in this sheet = Institute Affiliation Decl</t>
         </is>
@@ -2966,18 +3189,18 @@
       </c>
     </row>
     <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="62" t="inlineStr">
+      <c r="A3" s="56" t="inlineStr">
         <is>
           <t>D:\ai_doc_automation\Test Data\Institute Affiliation Declaration for Testing\Institute Declaration Certificate.pdf</t>
         </is>
       </c>
-      <c r="B3" s="63" t="inlineStr"/>
+      <c r="B3" s="57" t="inlineStr"/>
       <c r="C3" s="5" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
       </c>
-      <c r="D3" s="63" t="inlineStr"/>
+      <c r="D3" s="57" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2987,7 +3210,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00FCE4EC"/>
@@ -3004,7 +3227,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
-      <c r="A1" s="64" t="inlineStr">
+      <c r="A1" s="65" t="inlineStr">
         <is>
           <t>Paste full file paths in Column A (JPG / PNG / PDF). Column B = optional notes. Column C = Run Status (auto-updated by script). All files in this sheet = Orphan Certificate</t>
         </is>
@@ -3054,7 +3277,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00E0F2F1"/>
@@ -3071,7 +3294,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
-      <c r="A1" s="65" t="inlineStr">
+      <c r="A1" s="66" t="inlineStr">
         <is>
           <t>Paste full file paths in Column A (JPG / PNG / PDF). Column B = optional notes. Column C = Run Status (auto-updated by script). All files in this sheet = Ration Card</t>
         </is>
@@ -3100,32 +3323,997 @@
       </c>
     </row>
     <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="66" t="inlineStr">
+      <c r="A3" s="67" t="inlineStr">
         <is>
           <t>D:\ai_doc_automation\Test Data\Ration Card for Testing\Ration Card.pdf</t>
         </is>
       </c>
-      <c r="B3" s="67" t="inlineStr"/>
+      <c r="B3" s="68" t="inlineStr"/>
       <c r="C3" s="5" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
       </c>
-      <c r="D3" s="67" t="inlineStr"/>
+      <c r="D3" s="68" t="inlineStr"/>
     </row>
     <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="66" t="inlineStr">
+      <c r="A4" s="67" t="inlineStr">
         <is>
           <t>D:\ai_doc_automation\Test Data\Ration Card for Testing\ration.jpeg</t>
         </is>
       </c>
-      <c r="B4" s="67" t="inlineStr"/>
+      <c r="B4" s="68" t="inlineStr"/>
       <c r="C4" s="5" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
       </c>
-      <c r="D4" s="67" t="inlineStr"/>
+      <c r="D4" s="68" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00F3E5F5"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="65" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="36" customHeight="1">
+      <c r="A1" s="39" t="inlineStr">
+        <is>
+          <t>Paste full file paths in Column A (JPG / PNG / PDF). Column B = optional notes. Column C = Run Status (auto-updated by script). All files in this sheet = Divyang Certificate</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>File Path</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Notes (optional)</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Run Status</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Output Row</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="69" t="inlineStr">
+        <is>
+          <t>&lt;path to Divyang Certificate file 1&gt;</t>
+        </is>
+      </c>
+      <c r="B3" s="40" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D3" s="41" t="inlineStr"/>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="69" t="inlineStr">
+        <is>
+          <t>&lt;path to Divyang Certificate file 2&gt;</t>
+        </is>
+      </c>
+      <c r="B4" s="40" t="inlineStr"/>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D4" s="41" t="inlineStr"/>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="69" t="inlineStr">
+        <is>
+          <t>&lt;path to Divyang Certificate file 3&gt;</t>
+        </is>
+      </c>
+      <c r="B5" s="40" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D5" s="41" t="inlineStr"/>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="69" t="inlineStr">
+        <is>
+          <t>&lt;path to Divyang Certificate file 4&gt;</t>
+        </is>
+      </c>
+      <c r="B6" s="40" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D6" s="41" t="inlineStr"/>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="69" t="inlineStr">
+        <is>
+          <t>&lt;path to Divyang Certificate file 5&gt;</t>
+        </is>
+      </c>
+      <c r="B7" s="40" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D7" s="41" t="inlineStr"/>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="69" t="inlineStr">
+        <is>
+          <t>&lt;path to Divyang Certificate file 6&gt;</t>
+        </is>
+      </c>
+      <c r="B8" s="40" t="inlineStr"/>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D8" s="41" t="inlineStr"/>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="69" t="inlineStr">
+        <is>
+          <t>&lt;path to Divyang Certificate file 7&gt;</t>
+        </is>
+      </c>
+      <c r="B9" s="40" t="inlineStr"/>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D9" s="41" t="inlineStr"/>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="69" t="inlineStr">
+        <is>
+          <t>&lt;path to Divyang Certificate file 8&gt;</t>
+        </is>
+      </c>
+      <c r="B10" s="40" t="inlineStr"/>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D10" s="41" t="inlineStr"/>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="69" t="inlineStr">
+        <is>
+          <t>&lt;path to Divyang Certificate file 9&gt;</t>
+        </is>
+      </c>
+      <c r="B11" s="40" t="inlineStr"/>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D11" s="41" t="inlineStr"/>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="69" t="inlineStr">
+        <is>
+          <t>&lt;path to Divyang Certificate file 10&gt;</t>
+        </is>
+      </c>
+      <c r="B12" s="40" t="inlineStr"/>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D12" s="41" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00E0F7FA"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="65" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="36" customHeight="1">
+      <c r="A1" s="42" t="inlineStr">
+        <is>
+          <t>Paste full file paths in Column A (JPG / PNG / PDF). Column B = optional notes. Column C = Run Status (auto-updated by script). All files in this sheet = Occupation Certificate</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>File Path</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Notes (optional)</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Run Status</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Output Row</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="70" t="inlineStr">
+        <is>
+          <t>&lt;path to Occupation Certificate file 1&gt;</t>
+        </is>
+      </c>
+      <c r="B3" s="43" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D3" s="44" t="inlineStr"/>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="70" t="inlineStr">
+        <is>
+          <t>&lt;path to Occupation Certificate file 2&gt;</t>
+        </is>
+      </c>
+      <c r="B4" s="43" t="inlineStr"/>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D4" s="44" t="inlineStr"/>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="70" t="inlineStr">
+        <is>
+          <t>&lt;path to Occupation Certificate file 3&gt;</t>
+        </is>
+      </c>
+      <c r="B5" s="43" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D5" s="44" t="inlineStr"/>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="70" t="inlineStr">
+        <is>
+          <t>&lt;path to Occupation Certificate file 4&gt;</t>
+        </is>
+      </c>
+      <c r="B6" s="43" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D6" s="44" t="inlineStr"/>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="70" t="inlineStr">
+        <is>
+          <t>&lt;path to Occupation Certificate file 5&gt;</t>
+        </is>
+      </c>
+      <c r="B7" s="43" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D7" s="44" t="inlineStr"/>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="70" t="inlineStr">
+        <is>
+          <t>&lt;path to Occupation Certificate file 6&gt;</t>
+        </is>
+      </c>
+      <c r="B8" s="43" t="inlineStr"/>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D8" s="44" t="inlineStr"/>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="70" t="inlineStr">
+        <is>
+          <t>&lt;path to Occupation Certificate file 7&gt;</t>
+        </is>
+      </c>
+      <c r="B9" s="43" t="inlineStr"/>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D9" s="44" t="inlineStr"/>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="70" t="inlineStr">
+        <is>
+          <t>&lt;path to Occupation Certificate file 8&gt;</t>
+        </is>
+      </c>
+      <c r="B10" s="43" t="inlineStr"/>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D10" s="44" t="inlineStr"/>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="70" t="inlineStr">
+        <is>
+          <t>&lt;path to Occupation Certificate file 9&gt;</t>
+        </is>
+      </c>
+      <c r="B11" s="43" t="inlineStr"/>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D11" s="44" t="inlineStr"/>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="70" t="inlineStr">
+        <is>
+          <t>&lt;path to Occupation Certificate file 10&gt;</t>
+        </is>
+      </c>
+      <c r="B12" s="43" t="inlineStr"/>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D12" s="44" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00FBE9E7"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="65" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="36" customHeight="1">
+      <c r="A1" s="45" t="inlineStr">
+        <is>
+          <t>Paste full file paths in Column A (JPG / PNG / PDF). Column B = optional notes. Column C = Run Status (auto-updated by script). All files in this sheet = Annual Contribution Certificate</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>File Path</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Notes (optional)</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Run Status</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Output Row</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="71" t="inlineStr">
+        <is>
+          <t>&lt;path to Annual Contribution Certificate file 1&gt;</t>
+        </is>
+      </c>
+      <c r="B3" s="46" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D3" s="47" t="inlineStr"/>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="71" t="inlineStr">
+        <is>
+          <t>&lt;path to Annual Contribution Certificate file 2&gt;</t>
+        </is>
+      </c>
+      <c r="B4" s="46" t="inlineStr"/>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D4" s="47" t="inlineStr"/>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="71" t="inlineStr">
+        <is>
+          <t>&lt;path to Annual Contribution Certificate file 3&gt;</t>
+        </is>
+      </c>
+      <c r="B5" s="46" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D5" s="47" t="inlineStr"/>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="71" t="inlineStr">
+        <is>
+          <t>&lt;path to Annual Contribution Certificate file 4&gt;</t>
+        </is>
+      </c>
+      <c r="B6" s="46" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D6" s="47" t="inlineStr"/>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="71" t="inlineStr">
+        <is>
+          <t>&lt;path to Annual Contribution Certificate file 5&gt;</t>
+        </is>
+      </c>
+      <c r="B7" s="46" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D7" s="47" t="inlineStr"/>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="71" t="inlineStr">
+        <is>
+          <t>&lt;path to Annual Contribution Certificate file 6&gt;</t>
+        </is>
+      </c>
+      <c r="B8" s="46" t="inlineStr"/>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D8" s="47" t="inlineStr"/>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="71" t="inlineStr">
+        <is>
+          <t>&lt;path to Annual Contribution Certificate file 7&gt;</t>
+        </is>
+      </c>
+      <c r="B9" s="46" t="inlineStr"/>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D9" s="47" t="inlineStr"/>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="71" t="inlineStr">
+        <is>
+          <t>&lt;path to Annual Contribution Certificate file 8&gt;</t>
+        </is>
+      </c>
+      <c r="B10" s="46" t="inlineStr"/>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D10" s="47" t="inlineStr"/>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="71" t="inlineStr">
+        <is>
+          <t>&lt;path to Annual Contribution Certificate file 9&gt;</t>
+        </is>
+      </c>
+      <c r="B11" s="46" t="inlineStr"/>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D11" s="47" t="inlineStr"/>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="71" t="inlineStr">
+        <is>
+          <t>&lt;path to Annual Contribution Certificate file 10&gt;</t>
+        </is>
+      </c>
+      <c r="B12" s="46" t="inlineStr"/>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D12" s="47" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00E8F5E9"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="65" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="36" customHeight="1">
+      <c r="A1" s="48" t="inlineStr">
+        <is>
+          <t>Paste full file paths in Column A (JPG / PNG / PDF). Column B = optional notes. Column C = Run Status (auto-updated by script). All files in this sheet = Transgender Certificate</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>File Path</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Notes (optional)</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Run Status</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Output Row</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="72" t="inlineStr">
+        <is>
+          <t>&lt;path to Transgender Certificate file 1&gt;</t>
+        </is>
+      </c>
+      <c r="B3" s="49" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D3" s="50" t="inlineStr"/>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="72" t="inlineStr">
+        <is>
+          <t>&lt;path to Transgender Certificate file 2&gt;</t>
+        </is>
+      </c>
+      <c r="B4" s="49" t="inlineStr"/>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D4" s="50" t="inlineStr"/>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="72" t="inlineStr">
+        <is>
+          <t>&lt;path to Transgender Certificate file 3&gt;</t>
+        </is>
+      </c>
+      <c r="B5" s="49" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D5" s="50" t="inlineStr"/>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="72" t="inlineStr">
+        <is>
+          <t>&lt;path to Transgender Certificate file 4&gt;</t>
+        </is>
+      </c>
+      <c r="B6" s="49" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D6" s="50" t="inlineStr"/>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="72" t="inlineStr">
+        <is>
+          <t>&lt;path to Transgender Certificate file 5&gt;</t>
+        </is>
+      </c>
+      <c r="B7" s="49" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D7" s="50" t="inlineStr"/>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="72" t="inlineStr">
+        <is>
+          <t>&lt;path to Transgender Certificate file 6&gt;</t>
+        </is>
+      </c>
+      <c r="B8" s="49" t="inlineStr"/>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D8" s="50" t="inlineStr"/>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="72" t="inlineStr">
+        <is>
+          <t>&lt;path to Transgender Certificate file 7&gt;</t>
+        </is>
+      </c>
+      <c r="B9" s="49" t="inlineStr"/>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D9" s="50" t="inlineStr"/>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="72" t="inlineStr">
+        <is>
+          <t>&lt;path to Transgender Certificate file 8&gt;</t>
+        </is>
+      </c>
+      <c r="B10" s="49" t="inlineStr"/>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D10" s="50" t="inlineStr"/>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="72" t="inlineStr">
+        <is>
+          <t>&lt;path to Transgender Certificate file 9&gt;</t>
+        </is>
+      </c>
+      <c r="B11" s="49" t="inlineStr"/>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D11" s="50" t="inlineStr"/>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="72" t="inlineStr">
+        <is>
+          <t>&lt;path to Transgender Certificate file 10&gt;</t>
+        </is>
+      </c>
+      <c r="B12" s="49" t="inlineStr"/>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D12" s="50" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00EDE7F6"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="65" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="36" customHeight="1">
+      <c r="A1" s="51" t="inlineStr">
+        <is>
+          <t>Paste full file paths in Column A (JPG / PNG / PDF). Column B = optional notes. Column C = Run Status (auto-updated by script). All files in this sheet = Visa</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>File Path</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Notes (optional)</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Run Status</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Output Row</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="73" t="inlineStr">
+        <is>
+          <t>&lt;path to Visa file 1&gt;</t>
+        </is>
+      </c>
+      <c r="B3" s="52" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D3" s="53" t="inlineStr"/>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="73" t="inlineStr">
+        <is>
+          <t>&lt;path to Visa file 2&gt;</t>
+        </is>
+      </c>
+      <c r="B4" s="52" t="inlineStr"/>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D4" s="53" t="inlineStr"/>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="73" t="inlineStr">
+        <is>
+          <t>&lt;path to Visa file 3&gt;</t>
+        </is>
+      </c>
+      <c r="B5" s="52" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D5" s="53" t="inlineStr"/>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="73" t="inlineStr">
+        <is>
+          <t>&lt;path to Visa file 4&gt;</t>
+        </is>
+      </c>
+      <c r="B6" s="52" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D6" s="53" t="inlineStr"/>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="73" t="inlineStr">
+        <is>
+          <t>&lt;path to Visa file 5&gt;</t>
+        </is>
+      </c>
+      <c r="B7" s="52" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D7" s="53" t="inlineStr"/>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="73" t="inlineStr">
+        <is>
+          <t>&lt;path to Visa file 6&gt;</t>
+        </is>
+      </c>
+      <c r="B8" s="52" t="inlineStr"/>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D8" s="53" t="inlineStr"/>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="73" t="inlineStr">
+        <is>
+          <t>&lt;path to Visa file 7&gt;</t>
+        </is>
+      </c>
+      <c r="B9" s="52" t="inlineStr"/>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D9" s="53" t="inlineStr"/>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="73" t="inlineStr">
+        <is>
+          <t>&lt;path to Visa file 8&gt;</t>
+        </is>
+      </c>
+      <c r="B10" s="52" t="inlineStr"/>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D10" s="53" t="inlineStr"/>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="73" t="inlineStr">
+        <is>
+          <t>&lt;path to Visa file 9&gt;</t>
+        </is>
+      </c>
+      <c r="B11" s="52" t="inlineStr"/>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D11" s="53" t="inlineStr"/>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="73" t="inlineStr">
+        <is>
+          <t>&lt;path to Visa file 10&gt;</t>
+        </is>
+      </c>
+      <c r="B12" s="52" t="inlineStr"/>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="D12" s="53" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>